<commit_message>
cleaned up for presentation
</commit_message>
<xml_diff>
--- a/sim/CLEAN_alpha_outcomes.xlsx
+++ b/sim/CLEAN_alpha_outcomes.xlsx
@@ -1,20 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10419"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/riccardo/Desktop/Personal Projects/Latest/Yield curve models/gauss+/sim/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA67FCAA-417D-9B4C-BC25-992B5C05F772}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="240" yWindow="680" windowWidth="29160" windowHeight="15380" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="output" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
   <si>
     <t>Calibration outcomes for alpha</t>
   </si>
@@ -35,24 +41,6 @@
   </si>
   <si>
     <t>Alpha_l error</t>
-  </si>
-  <si>
-    <t>Sigma_m error (bps)</t>
-  </si>
-  <si>
-    <t>Sigma_l error (bps)</t>
-  </si>
-  <si>
-    <t>Rho error</t>
-  </si>
-  <si>
-    <t>avg. M factor error (bps)</t>
-  </si>
-  <si>
-    <t>avg. L factor error (bps)</t>
-  </si>
-  <si>
-    <t>Mu error (bps)</t>
   </si>
   <si>
     <t>Source: BSIC</t>
@@ -61,8 +49,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="5">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -114,7 +102,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="7">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -134,19 +122,6 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left style="thin">
         <color auto="1"/>
       </left>
@@ -194,30 +169,27 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -226,13 +198,21 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -270,7 +250,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -304,6 +284,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -338,9 +319,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -513,293 +495,150 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="B2:G17"/>
-  <sheetFormatPr defaultRowHeight="15.5" customHeight="1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="B2:G11"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15.5" customHeight="1" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="2" max="2" width="24.5" customWidth="1"/>
+    <col min="3" max="5" width="9" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="9.33203125" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="2" spans="2:7" ht="15.5" customHeight="1">
-      <c r="B2" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C2" s="1"/>
-      <c r="D2" s="1"/>
-      <c r="E2" s="1"/>
-      <c r="F2" s="1"/>
-      <c r="G2" s="1"/>
-    </row>
-    <row r="3" spans="2:7" ht="15.5" customHeight="1">
-      <c r="B3" s="2"/>
-      <c r="C3" s="2">
-        <v>0</v>
-      </c>
-      <c r="D3" s="2">
+    <row r="2" spans="2:7" ht="15.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B2" s="5"/>
+      <c r="C2" s="5"/>
+      <c r="D2" s="5"/>
+      <c r="E2" s="5"/>
+      <c r="F2" s="5"/>
+      <c r="G2" s="5"/>
+    </row>
+    <row r="3" spans="2:7" ht="15.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B3" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="C3" s="7"/>
+      <c r="D3" s="7"/>
+      <c r="E3" s="7"/>
+      <c r="F3" s="7"/>
+    </row>
+    <row r="4" spans="2:7" ht="15.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B4" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="E3" s="2">
+      <c r="C4" s="3">
+        <v>1.5</v>
+      </c>
+      <c r="D4" s="3">
+        <v>1.5</v>
+      </c>
+      <c r="E4" s="3">
+        <v>0.7</v>
+      </c>
+      <c r="F4" s="4">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="5" spans="2:7" ht="15.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B5" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="F3" s="2">
+      <c r="C5" s="3">
+        <v>1</v>
+      </c>
+      <c r="D5" s="3">
+        <v>0.85</v>
+      </c>
+      <c r="E5" s="3">
+        <v>0.4</v>
+      </c>
+      <c r="F5" s="4">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="6" spans="2:7" ht="15.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B6" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="G3" s="3">
+      <c r="C6" s="3">
+        <v>0.01</v>
+      </c>
+      <c r="D6" s="3">
+        <v>0.01</v>
+      </c>
+      <c r="E6" s="3">
+        <v>0.01</v>
+      </c>
+      <c r="F6" s="4">
+        <v>0.01</v>
+      </c>
+    </row>
+    <row r="7" spans="2:7" ht="15.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B7" s="1" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="4" spans="2:7" ht="15.5" customHeight="1">
-      <c r="B4" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="C4" s="5">
-        <v>1.5</v>
-      </c>
-      <c r="D4" s="5">
-        <v>1.5</v>
-      </c>
-      <c r="E4" s="5">
-        <v>1.5</v>
-      </c>
-      <c r="F4" s="5">
-        <v>0.7</v>
-      </c>
-      <c r="G4" s="6">
-        <v>0.7</v>
-      </c>
-    </row>
-    <row r="5" spans="2:7" ht="15.5" customHeight="1">
-      <c r="B5" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="C5" s="5">
-        <v>1</v>
-      </c>
-      <c r="D5" s="5">
-        <v>1</v>
-      </c>
-      <c r="E5" s="5">
-        <v>0.85</v>
-      </c>
-      <c r="F5" s="5">
-        <v>0.4</v>
-      </c>
-      <c r="G5" s="6">
-        <v>0.6</v>
-      </c>
-    </row>
-    <row r="6" spans="2:7" ht="15.5" customHeight="1">
-      <c r="B6" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="C6" s="5">
-        <v>0.01</v>
-      </c>
-      <c r="D6" s="5">
-        <v>0.017</v>
-      </c>
-      <c r="E6" s="5">
-        <v>0.01</v>
-      </c>
-      <c r="F6" s="5">
-        <v>0.01</v>
-      </c>
-      <c r="G6" s="6">
-        <v>0.01</v>
-      </c>
-    </row>
-    <row r="7" spans="2:7" ht="15.5" customHeight="1">
-      <c r="B7" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="C7" s="5">
+      <c r="C7" s="3">
         <v>-0.01</v>
       </c>
-      <c r="D7" s="5">
+      <c r="D7" s="3">
         <v>-0.01</v>
       </c>
-      <c r="E7" s="5">
-        <v>-0.01</v>
-      </c>
-      <c r="F7" s="5">
-        <v>0</v>
-      </c>
-      <c r="G7" s="6">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="2:7" ht="15.5" customHeight="1">
-      <c r="B8" s="4" t="s">
+      <c r="E7" s="3">
+        <v>0</v>
+      </c>
+      <c r="F7" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="2:7" ht="15.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B8" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C8" s="5">
-        <v>0.007</v>
-      </c>
-      <c r="D8" s="5">
-        <v>0.007</v>
-      </c>
-      <c r="E8" s="5">
-        <v>0.005</v>
-      </c>
-      <c r="F8" s="5">
-        <v>-0</v>
-      </c>
-      <c r="G8" s="6">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="2:7" ht="15.5" customHeight="1">
-      <c r="B9" s="4" t="s">
+      <c r="C8" s="3">
+        <v>7.0000000000000001E-3</v>
+      </c>
+      <c r="D8" s="3">
+        <v>5.0000000000000001E-3</v>
+      </c>
+      <c r="E8" s="3">
+        <v>0</v>
+      </c>
+      <c r="F8" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="2:7" ht="15.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B9" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C9" s="5">
-        <v>-0</v>
-      </c>
-      <c r="D9" s="5">
-        <v>-0</v>
-      </c>
-      <c r="E9" s="5">
-        <v>-0</v>
-      </c>
-      <c r="F9" s="5">
-        <v>0</v>
-      </c>
-      <c r="G9" s="6">
-        <v>-0</v>
-      </c>
-    </row>
-    <row r="10" spans="2:7" ht="15.5" customHeight="1">
-      <c r="B10" s="4" t="s">
+      <c r="C9" s="3">
+        <v>0</v>
+      </c>
+      <c r="D9" s="3">
+        <v>0</v>
+      </c>
+      <c r="E9" s="3">
+        <v>0</v>
+      </c>
+      <c r="F9" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="2:7" ht="5" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="11" spans="2:7" ht="15.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B11" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="C10" s="5">
-        <v>-96.39</v>
-      </c>
-      <c r="D10" s="5">
-        <v>-96.39</v>
-      </c>
-      <c r="E10" s="5">
-        <v>-96.39</v>
-      </c>
-      <c r="F10" s="5">
-        <v>-96.39</v>
-      </c>
-      <c r="G10" s="6">
-        <v>-96.39</v>
-      </c>
-    </row>
-    <row r="11" spans="2:7" ht="15.5" customHeight="1">
-      <c r="B11" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="C11" s="5">
-        <v>262.52</v>
-      </c>
-      <c r="D11" s="5">
-        <v>258.645</v>
-      </c>
-      <c r="E11" s="5">
-        <v>245.432</v>
-      </c>
-      <c r="F11" s="5">
-        <v>168.149</v>
-      </c>
-      <c r="G11" s="6">
-        <v>245.192</v>
-      </c>
-    </row>
-    <row r="12" spans="2:7" ht="15.5" customHeight="1">
-      <c r="B12" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="C12" s="5">
-        <v>-0.209</v>
-      </c>
-      <c r="D12" s="5">
-        <v>-0.208</v>
-      </c>
-      <c r="E12" s="5">
-        <v>-0.21</v>
-      </c>
-      <c r="F12" s="5">
-        <v>-0.211</v>
-      </c>
-      <c r="G12" s="6">
-        <v>-0.209</v>
-      </c>
-    </row>
-    <row r="13" spans="2:7" ht="15.5" customHeight="1">
-      <c r="B13" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="C13" s="5">
-        <v>-21.643</v>
-      </c>
-      <c r="D13" s="5">
-        <v>-19.063</v>
-      </c>
-      <c r="E13" s="5">
-        <v>-21.352</v>
-      </c>
-      <c r="F13" s="5">
-        <v>-13.588</v>
-      </c>
-      <c r="G13" s="6">
-        <v>-20.062</v>
-      </c>
-    </row>
-    <row r="14" spans="2:7" ht="15.5" customHeight="1">
-      <c r="B14" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="C14" s="5">
-        <v>29.834</v>
-      </c>
-      <c r="D14" s="5">
-        <v>26.731</v>
-      </c>
-      <c r="E14" s="5">
-        <v>34.952</v>
-      </c>
-      <c r="F14" s="5">
-        <v>52.459</v>
-      </c>
-      <c r="G14" s="6">
-        <v>50.696</v>
-      </c>
-    </row>
-    <row r="15" spans="2:7" ht="15.5" customHeight="1">
-      <c r="B15" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="C15" s="5">
-        <v>-759.95</v>
-      </c>
-      <c r="D15" s="5">
-        <v>-401.204</v>
-      </c>
-      <c r="E15" s="5">
-        <v>-842.253</v>
-      </c>
-      <c r="F15" s="5">
-        <v>-1065.465</v>
-      </c>
-      <c r="G15" s="6">
-        <v>-1070.986</v>
-      </c>
-    </row>
-    <row r="16" spans="2:7" ht="5" customHeight="1"/>
-    <row r="17" spans="2:7" ht="15.5" customHeight="1">
-      <c r="B17" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="C17" s="8"/>
-      <c r="D17" s="8"/>
-      <c r="E17" s="8"/>
-      <c r="F17" s="8"/>
-      <c r="G17" s="8"/>
+      <c r="C11" s="6"/>
+      <c r="D11" s="6"/>
+      <c r="E11" s="6"/>
+      <c r="F11" s="6"/>
+      <c r="G11" s="6"/>
     </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="3">
     <mergeCell ref="B2:G2"/>
-    <mergeCell ref="B17:G17"/>
+    <mergeCell ref="B11:G11"/>
+    <mergeCell ref="B3:F3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>